<commit_message>
filenames changes +partially T1697DNDtestcase
</commit_message>
<xml_diff>
--- a/TestData/LV_T1692_ValidationsToBeCompletedBeforeFVAOpportunityIsApproved.xlsx
+++ b/TestData/LV_T1692_ValidationsToBeCompletedBeforeFVAOpportunityIsApproved.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B21D3B-419E-48E2-8D82-42805527C91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82500FF-A812-49EF-9A8F-D41E0F758BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="93">
   <si>
     <t>Client</t>
   </si>
@@ -83,9 +83,6 @@
     <t>LegalEntity</t>
   </si>
   <si>
-    <t>HL Consulting, Inc.</t>
-  </si>
-  <si>
     <t>DisclosureStatus</t>
   </si>
   <si>
@@ -101,15 +98,6 @@
     <t>CaoUser</t>
   </si>
   <si>
-    <t>Retainer</t>
-  </si>
-  <si>
-    <t>MonthlyFee</t>
-  </si>
-  <si>
-    <t>ContingentFee</t>
-  </si>
-  <si>
     <t>ClientOwnership</t>
   </si>
   <si>
@@ -119,30 +107,9 @@
     <t>Public Equity</t>
   </si>
   <si>
-    <t>SICCode</t>
-  </si>
-  <si>
-    <t>OpportunityDescription</t>
-  </si>
-  <si>
     <t>Test</t>
   </si>
   <si>
-    <t>ReferralContact</t>
-  </si>
-  <si>
-    <t>Agreement</t>
-  </si>
-  <si>
-    <t>Yes, separate signed agreement</t>
-  </si>
-  <si>
-    <t>Outcome</t>
-  </si>
-  <si>
-    <t>Cleared</t>
-  </si>
-  <si>
     <t>Contact</t>
   </si>
   <si>
@@ -158,27 +125,12 @@
     <t>Party</t>
   </si>
   <si>
-    <t>RecordType</t>
-  </si>
-  <si>
-    <t>FASJobType</t>
-  </si>
-  <si>
-    <t>Consulting</t>
-  </si>
-  <si>
     <t>ClientType</t>
   </si>
   <si>
     <t>External</t>
   </si>
   <si>
-    <t>MarketCap</t>
-  </si>
-  <si>
-    <t>Fee</t>
-  </si>
-  <si>
     <t>Contact2</t>
   </si>
   <si>
@@ -326,12 +278,6 @@
     <t>Opportunity Detail - SIC Code., Opportunity Description - Opportunity Description., Estimated Financials - Est. Transaction Size/Market Cap., Estimated Fees - Retainer, input zero if there's no Retainer fee., Estimated Fees - Tail Expires., Estimated Fees - Progress/Monthly Fee., Estimated Fees - Contingent Fee., Referral Information - Referral Contact name is required., HL Internal Team - Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional)., Legal Matters - Confidentiality Agreement, Conflicts Check - A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed., Administration - Estimated Closed Date., Administration - "Women Led" is required. Please update this field with the correct value, Administration - Fairness Opinion Component., Administration - Date Engaged - Date of Executed Retainer or similar document., Approved NBC form - Please complete and submit this form via the NBC button., Opportunity Contacts - Add at least one Primary Opportunity Contact., Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>9999</t>
-  </si>
-  <si>
     <t>Estimated Financials - Client/Subject: EBITDA(MM), please provide a EBITDA(MM) value on the Client or Subject Company record in Company Financials</t>
   </si>
   <si>
@@ -350,26 +296,26 @@
     <t>Opportunities</t>
   </si>
   <si>
-    <t>FVA</t>
-  </si>
-  <si>
-    <t>Drew Koecher</t>
-  </si>
-  <si>
     <t>Dimitri Drone</t>
   </si>
   <si>
-    <t>10000</t>
-  </si>
-  <si>
     <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;General: SIC Code is required.Info--&gt;Details--&gt;General: Tombstone Permission is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: \"Women Led\" is required. Please update this field with the correct valueInfo--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved FEIS form - Please complete and submit this form via the FEIS button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.Opportunity Contacts - Add at least one Contact with an approrpriate Role - confirm with FVA BUAs.Info--&gt;Administration--&gt;Service &amp; Transaction Type: Transaction Type is required.Fees &amp; Financials--&gt;Estimated Fees: Total Anticipated Revenue is required.It should be Greater Than or Equal to the Fee.</t>
+  </si>
+  <si>
+    <t>Activism Advisory</t>
+  </si>
+  <si>
+    <t>HL Capital, Inc.</t>
+  </si>
+  <si>
+    <t>Rob Oudman</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -387,6 +333,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -412,14 +365,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -438,6 +389,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -718,11 +670,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
@@ -733,17 +684,11 @@
     <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.33203125" customWidth="1"/>
+    <col min="15" max="15" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -781,63 +726,27 @@
         <v>16</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="O1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -864,55 +773,19 @@
         <v>15</v>
       </c>
       <c r="L2" t="s">
-        <v>17</v>
+        <v>91</v>
       </c>
       <c r="M2" t="s">
-        <v>19</v>
-      </c>
-      <c r="N2" t="s">
-        <v>107</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>98</v>
+        <v>18</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>92</v>
       </c>
       <c r="R2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="S2" t="s">
-        <v>28</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="U2" t="s">
-        <v>31</v>
-      </c>
-      <c r="V2" t="s">
-        <v>95</v>
-      </c>
-      <c r="W2" t="s">
-        <v>34</v>
-      </c>
-      <c r="X2" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AB2" s="3" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -932,15 +805,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -958,12 +831,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -978,12 +851,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1008,76 +881,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="162" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="162" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="8" t="s">
+      <c r="D2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G2" s="8" t="s">
+      <c r="F2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>100</v>
+      <c r="H2" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1091,318 +964,318 @@
   <dimension ref="A1:AF33"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="95.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="8" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" style="8"/>
-    <col min="8" max="8" width="12.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="12" width="8.88671875" style="8"/>
-    <col min="13" max="13" width="10.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.88671875" style="3"/>
-    <col min="15" max="16" width="8.88671875" style="8"/>
-    <col min="17" max="17" width="10.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="29.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="8.88671875" style="8"/>
-    <col min="21" max="21" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.88671875" style="8"/>
-    <col min="23" max="23" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="30" width="8.88671875" style="8"/>
-    <col min="31" max="31" width="10.5546875" style="8" customWidth="1"/>
-    <col min="32" max="32" width="102.33203125" style="8" customWidth="1"/>
-    <col min="33" max="16384" width="8.88671875" style="8"/>
+    <col min="1" max="1" width="95.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="6"/>
+    <col min="8" max="8" width="12.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="12" width="8.88671875" style="6"/>
+    <col min="13" max="13" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.88671875" style="2"/>
+    <col min="15" max="16" width="8.88671875" style="6"/>
+    <col min="17" max="17" width="10.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="8.88671875" style="6"/>
+    <col min="21" max="21" width="9.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8.88671875" style="6"/>
+    <col min="23" max="23" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="24" max="30" width="8.88671875" style="6"/>
+    <col min="31" max="31" width="10.5546875" style="6" customWidth="1"/>
+    <col min="32" max="32" width="102.33203125" style="6" customWidth="1"/>
+    <col min="33" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:32" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="P1" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="Q1" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="R1" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="S1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="T1" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="U1" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="X1" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC1" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="AD1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="AE1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AF1" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" ht="216" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="R1" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="S1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="T1" s="9" t="s">
+      <c r="K2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AA2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF2" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="U1" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="V1" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="W1" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="X1" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="Y1" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="Z1" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA1" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="AB1" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AC1" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="AD1" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="AE1" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="AF1" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:32" ht="216" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="R2" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="S2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="X2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AA2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AB2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AD2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="AF2" s="7" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
+      <c r="A3" s="3"/>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
+      <c r="A4" s="3"/>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
+      <c r="A5" s="3"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
+      <c r="A6" s="3"/>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
+      <c r="A7" s="3"/>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
+      <c r="A8" s="3"/>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
+      <c r="A9" s="3"/>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
+      <c r="A10" s="3"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
+      <c r="A11" s="3"/>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
+      <c r="A12" s="3"/>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
+      <c r="A13" s="3"/>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
+      <c r="A14" s="3"/>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
+      <c r="A15" s="3"/>
     </row>
     <row r="16" spans="1:32" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
+      <c r="A16" s="3"/>
     </row>
     <row r="17" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
+      <c r="A17" s="3"/>
     </row>
     <row r="18" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
+      <c r="A18" s="3"/>
     </row>
     <row r="19" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
+      <c r="A19" s="3"/>
     </row>
     <row r="20" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
+      <c r="A20" s="3"/>
     </row>
     <row r="21" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
+      <c r="A21" s="3"/>
     </row>
     <row r="22" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
+      <c r="A22" s="3"/>
     </row>
     <row r="23" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
+      <c r="A23" s="3"/>
     </row>
     <row r="24" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
+      <c r="A24" s="3"/>
     </row>
     <row r="25" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
+      <c r="A25" s="3"/>
     </row>
     <row r="26" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="5"/>
+      <c r="A26" s="3"/>
     </row>
     <row r="27" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="5"/>
+      <c r="A27" s="3"/>
     </row>
     <row r="28" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
+      <c r="A28" s="3"/>
     </row>
     <row r="29" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
+      <c r="A29" s="3"/>
     </row>
     <row r="30" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="5"/>
+      <c r="A30" s="3"/>
     </row>
     <row r="31" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="5"/>
+      <c r="A31" s="3"/>
     </row>
     <row r="32" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="5"/>
+      <c r="A32" s="3"/>
     </row>
     <row r="33" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="5"/>
+      <c r="A33" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>